<commit_message>
Add project presentation and typographic styles for e-commerce AI assistant
- Created a new PowerPoint presentation file for the project defense titled "电商 AI 商品文案生成与智能导购助手".
- Added a new typographic file defining styles and components for the presentation, including color schemes, text styles, and layout structures.
- Included sections covering project objectives, system architecture, AI capabilities, and team contributions.
</commit_message>
<xml_diff>
--- a/frontend/submission-output/项目组成员分工-本项目.xlsx
+++ b/frontend/submission-output/项目组成员分工-本项目.xlsx
@@ -13,6 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'项目组成员分工'!$A$5:$H$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'项目组成员分工'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'模块责任矩阵'!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -70,7 +71,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +86,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -155,16 +161,17 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -853,7 +860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -872,330 +879,384 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="12" t="n"/>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="12" t="n"/>
+      <c r="G2" s="12" t="n"/>
+    </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>模块</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>前端1</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>前端2</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>后端</t>
         </is>
       </c>
-      <c r="F3" s="12" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>数据/AI</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>测试/文档</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>需求与计划</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>用户端</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>商家端</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>认证与 API</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>数据库与迁移</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr"/>
-      <c r="D8" s="13" t="inlineStr"/>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>AI 与 RAG</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>测试与部署</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>文档与答辩</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>